<commit_message>
BUG FIX site status related DateEntry colour and value assignment.
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template__COPY.xlsx
+++ b/rss_islandr/templates/report_template__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="53">
   <si>
     <t>Soil</t>
   </si>
@@ -143,21 +143,6 @@
     <t>Coordinates (lat-lng)</t>
   </si>
   <si>
-    <t>Giorgos Makris Industry</t>
-  </si>
-  <si>
-    <t>Airports (NACE Code H.52.23)</t>
-  </si>
-  <si>
-    <t>Artificial Surfaces - Artificial, non-agricultural vegetated areas</t>
-  </si>
-  <si>
-    <t>Legacy</t>
-  </si>
-  <si>
-    <t>CLAY - silty clay</t>
-  </si>
-  <si>
     <t>Bio-accumulative and toxic materials</t>
   </si>
   <si>
@@ -173,43 +158,34 @@
     <t>No limit to access</t>
   </si>
   <si>
-    <t>&gt;=3m</t>
-  </si>
-  <si>
-    <t>None</t>
+    <t>&lt;1m</t>
   </si>
   <si>
     <t>Unconfined</t>
   </si>
   <si>
-    <t>Silt/clay aquifer: 20m</t>
+    <t>Silt/clay aquifer: 100m</t>
   </si>
   <si>
     <t>Area source</t>
   </si>
   <si>
-    <t>&lt;1km</t>
-  </si>
-  <si>
-    <t>PM10</t>
-  </si>
-  <si>
-    <t>Frequent</t>
-  </si>
-  <si>
-    <t>Sand</t>
-  </si>
-  <si>
-    <t>Residential</t>
-  </si>
-  <si>
-    <t>Irrigation</t>
-  </si>
-  <si>
-    <t>Domestic/potable</t>
-  </si>
-  <si>
-    <t>Option 2</t>
+    <t>1km-5km</t>
+  </si>
+  <si>
+    <t>PM2.5</t>
+  </si>
+  <si>
+    <t>Value Not Known</t>
+  </si>
+  <si>
+    <t>Industrial</t>
+  </si>
+  <si>
+    <t>Significant waterway</t>
+  </si>
+  <si>
+    <t>Option 1</t>
   </si>
 </sst>
 </file>
@@ -880,27 +856,21 @@
         <v>2</v>
       </c>
       <c r="B2" s="21"/>
-      <c r="C2" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="21" t="s">
         <v>31</v>
       </c>
       <c r="G2" s="21"/>
-      <c r="H2" s="3" t="s">
-        <v>39</v>
-      </c>
+      <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="24" t="s">
         <v>34</v>
       </c>
       <c r="L2" s="24"/>
-      <c r="M2" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
@@ -909,27 +879,21 @@
         <v>30</v>
       </c>
       <c r="B3" s="16"/>
-      <c r="C3" s="9">
-        <v>45720</v>
-      </c>
+      <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="16" t="s">
         <v>32</v>
       </c>
       <c r="G3" s="16"/>
-      <c r="H3" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="16" t="s">
         <v>35</v>
       </c>
       <c r="L3" s="16"/>
-      <c r="M3" s="9">
-        <v>45734</v>
-      </c>
+      <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
@@ -939,28 +903,24 @@
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="15">
-        <v>48.341650000000001</v>
+        <v>0</v>
       </c>
       <c r="D4" s="15">
-        <v>10.195309999999999</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="23" t="s">
         <v>33</v>
       </c>
       <c r="G4" s="23"/>
-      <c r="H4" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="23" t="s">
         <v>36</v>
       </c>
       <c r="L4" s="23"/>
-      <c r="M4" s="9">
-        <v>45741</v>
-      </c>
+      <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
@@ -989,7 +949,7 @@
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1010,7 +970,7 @@
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1031,7 +991,7 @@
       </c>
       <c r="B8" s="22"/>
       <c r="C8" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1051,9 +1011,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="22"/>
-      <c r="C9" s="5">
-        <v>1</v>
-      </c>
+      <c r="C9" s="5"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1119,35 +1077,35 @@
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="E12" s="21"/>
       <c r="F12" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="K12" s="21"/>
       <c r="L12" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="M12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="N12" s="21"/>
       <c r="O12" s="7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1156,35 +1114,35 @@
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>11</v>
       </c>
       <c r="H13" s="16"/>
       <c r="I13" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>21</v>
       </c>
       <c r="N13" s="16"/>
       <c r="O13" s="7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1193,35 +1151,35 @@
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>17</v>
       </c>
       <c r="H14" s="16"/>
       <c r="I14" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>19</v>
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>22</v>
       </c>
       <c r="N14" s="16"/>
       <c r="O14" s="7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1230,33 +1188,31 @@
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
-      <c r="I15" s="5">
-        <v>1</v>
-      </c>
+      <c r="I15" s="5"/>
       <c r="J15" s="16" t="s">
         <v>20</v>
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>23</v>
       </c>
       <c r="N15" s="16"/>
       <c r="O15" s="7" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1265,26 +1221,20 @@
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
-      <c r="F16" s="5">
-        <v>1</v>
-      </c>
+      <c r="F16" s="5"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="6"/>
       <c r="J16" s="16"/>
       <c r="K16" s="16"/>
-      <c r="L16" s="5">
-        <v>1</v>
-      </c>
+      <c r="L16" s="5"/>
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
-      <c r="O16" s="8">
-        <v>0.6</v>
-      </c>
+      <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
@@ -1292,28 +1242,36 @@
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="12">
-        <v>0.35</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="16"/>
-      <c r="F17" s="13"/>
+      <c r="F17" s="13">
+        <v>0.14699999999999899</v>
+      </c>
       <c r="G17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="H17" s="16"/>
-      <c r="I17" s="13"/>
+      <c r="I17" s="13">
+        <v>0.7</v>
+      </c>
       <c r="J17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="K17" s="16"/>
-      <c r="L17" s="13"/>
+      <c r="L17" s="13">
+        <v>0.29399999999999898</v>
+      </c>
       <c r="M17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="N17" s="16"/>
-      <c r="O17" s="14"/>
+      <c r="O17" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
@@ -1409,35 +1367,35 @@
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="4" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="4" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="4" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="K21" s="16"/>
       <c r="L21" s="4" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="M21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="16"/>
       <c r="O21" s="7" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1446,35 +1404,35 @@
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="11">
-        <v>0.17499999999999999</v>
+        <v>0.244999999999999</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="11">
-        <v>0.17499999999999999</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="11">
-        <v>0.35</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="K22" s="16"/>
       <c r="L22" s="11">
-        <v>0.105</v>
+        <v>0.14699999999999899</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="N22" s="16"/>
       <c r="O22" s="10">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementation of nested comboboxes
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template__COPY.xlsx
+++ b/rss_islandr/templates/report_template__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
   <si>
     <t>Soil</t>
   </si>
@@ -143,19 +143,25 @@
     <t>Coordinates (lat-lng)</t>
   </si>
   <si>
-    <t>helsinki</t>
-  </si>
-  <si>
-    <t>Airports (NACE Code H.52.23)</t>
-  </si>
-  <si>
-    <t>Artificial Surfaces - Mine, dump and construction sites</t>
-  </si>
-  <si>
-    <t>Legacy</t>
-  </si>
-  <si>
-    <t>CLAY - sandy clay</t>
+    <t>My scenario</t>
+  </si>
+  <si>
+    <t>Abrasive blasting (NACE Code C.28.49)</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Clay</t>
+  </si>
+  <si>
+    <t>Sandy clay</t>
+  </si>
+  <si>
+    <t>Forests and semi natural areas</t>
+  </si>
+  <si>
+    <t>Scrub and/or herbaceous vegetation associations</t>
   </si>
   <si>
     <t>Bio-accumulative and toxic materials</t>
@@ -167,19 +173,37 @@
     <t>High</t>
   </si>
   <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Limited access</t>
+  </si>
+  <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Limited access</t>
-  </si>
-  <si>
     <t>2m</t>
   </si>
   <si>
-    <t>Value Not Known</t>
+    <t>5m</t>
+  </si>
+  <si>
+    <t>Silt/clay aquifer: 50m</t>
+  </si>
+  <si>
+    <t>Area source</t>
+  </si>
+  <si>
+    <t>&lt;1km</t>
+  </si>
+  <si>
+    <t>PM2.5</t>
+  </si>
+  <si>
+    <t>Frequent</t>
+  </si>
+  <si>
+    <t>Sand</t>
   </si>
   <si>
     <t>Industrial</t>
@@ -878,7 +902,7 @@
       </c>
       <c r="L2" s="24"/>
       <c r="M2" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
@@ -889,7 +913,7 @@
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="9">
-        <v>45719</v>
+        <v>45721</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -898,16 +922,18 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="J3" s="1"/>
       <c r="K3" s="16" t="s">
         <v>35</v>
       </c>
       <c r="L3" s="16"/>
       <c r="M3" s="9">
-        <v>45721</v>
+        <v>33665</v>
       </c>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
@@ -918,10 +944,10 @@
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="15">
-        <v>59.9330004237463</v>
+        <v>48.806863461085101</v>
       </c>
       <c r="D4" s="15">
-        <v>25.048828125</v>
+        <v>12.392578125</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="23" t="s">
@@ -929,17 +955,17 @@
       </c>
       <c r="G4" s="23"/>
       <c r="H4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="23" t="s">
         <v>36</v>
       </c>
       <c r="L4" s="23"/>
-      <c r="M4" s="9">
-        <v>45729</v>
-      </c>
+      <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
@@ -968,7 +994,7 @@
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -989,7 +1015,7 @@
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1010,7 +1036,7 @@
       </c>
       <c r="B8" s="22"/>
       <c r="C8" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1098,14 +1124,14 @@
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="E12" s="21"/>
       <c r="F12" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>5</v>
@@ -1119,14 +1145,14 @@
       </c>
       <c r="K12" s="21"/>
       <c r="L12" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="M12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="N12" s="21"/>
       <c r="O12" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1135,7 +1161,7 @@
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>11</v>
@@ -1156,14 +1182,14 @@
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>21</v>
       </c>
       <c r="N13" s="16"/>
       <c r="O13" s="7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1172,35 +1198,35 @@
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>17</v>
       </c>
       <c r="H14" s="16"/>
       <c r="I14" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>19</v>
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>22</v>
       </c>
       <c r="N14" s="16"/>
       <c r="O14" s="7" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1209,14 +1235,14 @@
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -1226,14 +1252,14 @@
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>23</v>
       </c>
       <c r="N15" s="16"/>
       <c r="O15" s="7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1242,7 +1268,7 @@
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -1263,35 +1289,35 @@
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="12">
-        <v>0.3584</v>
+        <v>0.51200000000000001</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13">
-        <v>0</v>
+        <v>0.33599999999999902</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="13">
-        <v>0</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="K17" s="16"/>
       <c r="L17" s="13">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="M17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="N17" s="16"/>
       <c r="O17" s="14">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
@@ -1388,35 +1414,35 @@
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="4" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="4" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="4" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="K21" s="16"/>
       <c r="L21" s="4" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="M21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="16"/>
       <c r="O21" s="7" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1425,35 +1451,35 @@
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="11">
-        <v>0.1792</v>
+        <v>0.25600000000000001</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="11">
-        <v>0.3584</v>
+        <v>0.51200000000000001</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="11">
-        <v>0.3584</v>
+        <v>0.51200000000000001</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="K22" s="16"/>
       <c r="L22" s="11">
-        <v>0.10751999999999901</v>
+        <v>0.15359999999999999</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="N22" s="16"/>
       <c r="O22" s="10">
-        <v>0</v>
+        <v>0.14699999999999899</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed legends and other minor changes
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template__COPY.xlsx
+++ b/rss_islandr/templates/report_template__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="61">
   <si>
     <t>Soil</t>
   </si>
@@ -143,13 +143,13 @@
     <t>Coordinates (lat-lng)</t>
   </si>
   <si>
-    <t>My scenario</t>
-  </si>
-  <si>
-    <t>Abrasive blasting (NACE Code C.28.49)</t>
-  </si>
-  <si>
-    <t>Active</t>
+    <t>Oslo site</t>
+  </si>
+  <si>
+    <t>Airports (NACE Code H.52.23)</t>
+  </si>
+  <si>
+    <t>Legacy</t>
   </si>
   <si>
     <t>Clay</t>
@@ -158,10 +158,10 @@
     <t>Sandy clay</t>
   </si>
   <si>
-    <t>Forests and semi natural areas</t>
-  </si>
-  <si>
-    <t>Scrub and/or herbaceous vegetation associations</t>
+    <t>Agricultural areas</t>
+  </si>
+  <si>
+    <t>Permanent crops</t>
   </si>
   <si>
     <t>Bio-accumulative and toxic materials</t>
@@ -176,19 +176,16 @@
     <t>None</t>
   </si>
   <si>
-    <t>Limited access</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>2m</t>
-  </si>
-  <si>
-    <t>5m</t>
-  </si>
-  <si>
-    <t>Silt/clay aquifer: 50m</t>
+    <t>No limit to access</t>
+  </si>
+  <si>
+    <t>&lt;1m</t>
+  </si>
+  <si>
+    <t>Unconfined</t>
+  </si>
+  <si>
+    <t>Silt/clay aquifer: 20m</t>
   </si>
   <si>
     <t>Area source</t>
@@ -197,13 +194,13 @@
     <t>&lt;1km</t>
   </si>
   <si>
-    <t>PM2.5</t>
+    <t>PM10</t>
   </si>
   <si>
     <t>Frequent</t>
   </si>
   <si>
-    <t>Sand</t>
+    <t>Gravel</t>
   </si>
   <si>
     <t>Industrial</t>
@@ -933,7 +930,7 @@
       </c>
       <c r="L3" s="16"/>
       <c r="M3" s="9">
-        <v>33665</v>
+        <v>45078</v>
       </c>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
@@ -944,10 +941,10 @@
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="15">
-        <v>48.806863461085101</v>
+        <v>59.712097173322903</v>
       </c>
       <c r="D4" s="15">
-        <v>12.392578125</v>
+        <v>11.162109375</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="23" t="s">
@@ -965,7 +962,9 @@
         <v>36</v>
       </c>
       <c r="L4" s="23"/>
-      <c r="M4" s="9"/>
+      <c r="M4" s="9">
+        <v>45721</v>
+      </c>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
@@ -1138,7 +1137,7 @@
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J12" s="21" t="s">
         <v>5</v>
@@ -1168,21 +1167,21 @@
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>11</v>
       </c>
       <c r="H13" s="16"/>
       <c r="I13" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>21</v>
@@ -1205,7 +1204,7 @@
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>17</v>
@@ -1219,14 +1218,14 @@
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>22</v>
       </c>
       <c r="N14" s="16"/>
       <c r="O14" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1235,14 +1234,14 @@
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -1252,14 +1251,14 @@
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>23</v>
       </c>
       <c r="N15" s="16"/>
       <c r="O15" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1268,7 +1267,7 @@
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -1289,35 +1288,35 @@
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="12">
-        <v>0.51200000000000001</v>
+        <v>1</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13">
-        <v>0.33599999999999902</v>
+        <v>1</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="13">
-        <v>0.48999999999999899</v>
+        <v>1</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="K17" s="16"/>
       <c r="L17" s="13">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="M17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="N17" s="16"/>
       <c r="O17" s="14">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
@@ -1414,35 +1413,35 @@
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="K21" s="16"/>
       <c r="L21" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="16"/>
       <c r="O21" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1451,35 +1450,35 @@
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="11">
-        <v>0.25600000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="11">
-        <v>0.51200000000000001</v>
+        <v>1</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="11">
-        <v>0.51200000000000001</v>
+        <v>1</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="K22" s="16"/>
       <c r="L22" s="11">
-        <v>0.15359999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="N22" s="16"/>
       <c r="O22" s="10">
-        <v>0.14699999999999899</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DateEntry widget values are updated when scenario is imported
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template__COPY.xlsx
+++ b/rss_islandr/templates/report_template__COPY.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="46">
   <si>
     <t>Soil</t>
   </si>
@@ -143,64 +143,19 @@
     <t>Coordinates (lat-lng)</t>
   </si>
   <si>
-    <t>Oslo site</t>
-  </si>
-  <si>
-    <t>Airports (NACE Code H.52.23)</t>
-  </si>
-  <si>
-    <t>Legacy</t>
-  </si>
-  <si>
-    <t>Clay</t>
-  </si>
-  <si>
-    <t>Sandy clay</t>
-  </si>
-  <si>
-    <t>Agricultural areas</t>
-  </si>
-  <si>
-    <t>Permanent crops</t>
-  </si>
-  <si>
-    <t>Bio-accumulative and toxic materials</t>
-  </si>
-  <si>
-    <t>Large</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>No limit to access</t>
-  </si>
-  <si>
-    <t>&lt;1m</t>
-  </si>
-  <si>
-    <t>Unconfined</t>
-  </si>
-  <si>
-    <t>Silt/clay aquifer: 20m</t>
-  </si>
-  <si>
-    <t>Area source</t>
-  </si>
-  <si>
-    <t>&lt;1km</t>
-  </si>
-  <si>
-    <t>PM10</t>
-  </si>
-  <si>
-    <t>Frequent</t>
-  </si>
-  <si>
-    <t>Gravel</t>
+    <t>Silt</t>
+  </si>
+  <si>
+    <t>Clayey silt</t>
+  </si>
+  <si>
+    <t>Artificial surfaces</t>
+  </si>
+  <si>
+    <t>Urban fabric</t>
+  </si>
+  <si>
+    <t>Value Not Known</t>
   </si>
   <si>
     <t>Industrial</t>
@@ -880,27 +835,21 @@
         <v>2</v>
       </c>
       <c r="B2" s="21"/>
-      <c r="C2" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="21" t="s">
         <v>31</v>
       </c>
       <c r="G2" s="21"/>
-      <c r="H2" s="3" t="s">
-        <v>39</v>
-      </c>
+      <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="24" t="s">
         <v>34</v>
       </c>
       <c r="L2" s="24"/>
-      <c r="M2" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
@@ -909,9 +858,7 @@
         <v>30</v>
       </c>
       <c r="B3" s="16"/>
-      <c r="C3" s="9">
-        <v>45721</v>
-      </c>
+      <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="16" t="s">
@@ -919,19 +866,17 @@
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="16" t="s">
         <v>35</v>
       </c>
       <c r="L3" s="16"/>
-      <c r="M3" s="9">
-        <v>45078</v>
-      </c>
+      <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
@@ -941,10 +886,10 @@
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="15">
-        <v>59.712097173322903</v>
+        <v>0</v>
       </c>
       <c r="D4" s="15">
-        <v>11.162109375</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="23" t="s">
@@ -952,19 +897,17 @@
       </c>
       <c r="G4" s="23"/>
       <c r="H4" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="23" t="s">
         <v>36</v>
       </c>
       <c r="L4" s="23"/>
-      <c r="M4" s="9">
-        <v>45721</v>
-      </c>
+      <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
@@ -993,7 +936,7 @@
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1014,7 +957,7 @@
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1035,7 +978,7 @@
       </c>
       <c r="B8" s="22"/>
       <c r="C8" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1056,7 +999,7 @@
       </c>
       <c r="B9" s="22"/>
       <c r="C9" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1123,35 +1066,35 @@
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="E12" s="21"/>
       <c r="F12" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="21"/>
       <c r="I12" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="K12" s="21"/>
       <c r="L12" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="M12" s="21" t="s">
         <v>5</v>
       </c>
       <c r="N12" s="21"/>
       <c r="O12" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1160,35 +1103,35 @@
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>11</v>
       </c>
       <c r="H13" s="16"/>
       <c r="I13" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="4" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>21</v>
       </c>
       <c r="N13" s="16"/>
       <c r="O13" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1197,35 +1140,35 @@
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="4" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>17</v>
       </c>
       <c r="H14" s="16"/>
       <c r="I14" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>19</v>
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="4" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>22</v>
       </c>
       <c r="N14" s="16"/>
       <c r="O14" s="7" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1234,14 +1177,14 @@
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="4" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="G15" s="16"/>
       <c r="H15" s="16"/>
@@ -1251,14 +1194,14 @@
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="4" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="M15" s="16" t="s">
         <v>23</v>
       </c>
       <c r="N15" s="16"/>
       <c r="O15" s="7" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1267,7 +1210,7 @@
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="4" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -1288,35 +1231,35 @@
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="K17" s="16"/>
       <c r="L17" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" s="16" t="s">
         <v>6</v>
       </c>
       <c r="N17" s="16"/>
       <c r="O17" s="14">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
@@ -1413,35 +1356,35 @@
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="4" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="4" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="H21" s="16"/>
       <c r="I21" s="4" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="K21" s="16"/>
       <c r="L21" s="4" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="M21" s="16" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="16"/>
       <c r="O21" s="7" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1450,35 +1393,35 @@
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="H22" s="16"/>
       <c r="I22" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="K22" s="16"/>
       <c r="L22" s="11">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="M22" s="16" t="s">
         <v>27</v>
       </c>
       <c r="N22" s="16"/>
       <c r="O22" s="10">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>